<commit_message>
Publish portfolio PDF Word Excel and saved Yahoo evidence
</commit_message>
<xml_diff>
--- a/portfolio_construction/Portfolio Final/Results.xlsx
+++ b/portfolio_construction/Portfolio Final/Results.xlsx
@@ -995,10 +995,10 @@
         </is>
       </c>
       <c r="D31">
-        <v>0.1372476690650974</v>
+        <v>0.1372476690650976</v>
       </c>
       <c r="E31">
-        <v>854949.5969144428</v>
+        <v>854949.5969144441</v>
       </c>
     </row>
     <row r="32">
@@ -1087,10 +1087,10 @@
         </is>
       </c>
       <c r="D35">
-        <v>0.1127523309349027</v>
+        <v>0.1127523309349023</v>
       </c>
       <c r="E35">
-        <v>702362.091397246</v>
+        <v>702362.0913972433</v>
       </c>
     </row>
     <row r="36">
@@ -1179,10 +1179,10 @@
         </is>
       </c>
       <c r="D39">
-        <v>0.0979014944789439</v>
+        <v>0.09790149447894382</v>
       </c>
       <c r="E39">
-        <v>609852.5666209663</v>
+        <v>609852.5666209657</v>
       </c>
     </row>
     <row r="40">
@@ -1274,7 +1274,7 @@
         <v>0.1069382666493139</v>
       </c>
       <c r="E43">
-        <v>666144.8503230744</v>
+        <v>666144.850323074</v>
       </c>
     </row>
     <row r="44">
@@ -1320,7 +1320,7 @@
         <v>0.15</v>
       </c>
       <c r="E45">
-        <v>934387.0129870129</v>
+        <v>934387.012987013</v>
       </c>
     </row>
     <row r="46">
@@ -1409,10 +1409,10 @@
         </is>
       </c>
       <c r="D49">
-        <v>0.04516023887174229</v>
+        <v>0.04516023887174237</v>
       </c>
       <c r="E49">
-        <v>281314.2713676485</v>
+        <v>281314.271367649</v>
       </c>
     </row>
     <row r="50">
@@ -1478,10 +1478,10 @@
         </is>
       </c>
       <c r="D52">
-        <v>0.04391359239887407</v>
+        <v>0.04391359239887393</v>
       </c>
       <c r="E52">
-        <v>273548.6028740876</v>
+        <v>273548.6028740867</v>
       </c>
     </row>
     <row r="53">
@@ -1550,7 +1550,7 @@
         <v>0.1393715969982425</v>
       </c>
       <c r="E55">
-        <v>868180.0680961171</v>
+        <v>868180.0680961172</v>
       </c>
     </row>
     <row r="56">
@@ -1616,10 +1616,10 @@
         </is>
       </c>
       <c r="D58">
-        <v>0.0001758333460199443</v>
+        <v>0.0001758333460199342</v>
       </c>
       <c r="E58">
-        <v>1095.309299807251</v>
+        <v>1095.309299807188</v>
       </c>
     </row>
     <row r="59">
@@ -1639,10 +1639,10 @@
         </is>
       </c>
       <c r="D59">
-        <v>0.07708630041242337</v>
+        <v>0.07708630041242333</v>
       </c>
       <c r="E59">
-        <v>480189.5865638921</v>
+        <v>480189.5865638919</v>
       </c>
     </row>
     <row r="60">
@@ -2007,10 +2007,10 @@
         </is>
       </c>
       <c r="D75">
-        <v>0.15</v>
+        <v>0.1499999999999999</v>
       </c>
       <c r="E75">
-        <v>931434.3656343658</v>
+        <v>931434.3656343655</v>
       </c>
     </row>
     <row r="76">
@@ -2030,10 +2030,10 @@
         </is>
       </c>
       <c r="D76">
-        <v>0.04257117849736252</v>
+        <v>0.04257117849736258</v>
       </c>
       <c r="E76">
-        <v>264348.3909199881</v>
+        <v>264348.3909199885</v>
       </c>
     </row>
     <row r="77">
@@ -2076,10 +2076,10 @@
         </is>
       </c>
       <c r="D78">
-        <v>0.09048938186563894</v>
+        <v>0.09048938186563847</v>
       </c>
       <c r="E78">
-        <v>561899.4666311153</v>
+        <v>561899.4666311124</v>
       </c>
     </row>
     <row r="79">
@@ -2099,10 +2099,10 @@
         </is>
       </c>
       <c r="D79">
-        <v>0.1419467823439489</v>
+        <v>0.1419467823439498</v>
       </c>
       <c r="E79">
-        <v>881427.4077758364</v>
+        <v>881427.4077758415</v>
       </c>
     </row>
     <row r="80">
@@ -2148,7 +2148,7 @@
         <v>0.1254882653443414</v>
       </c>
       <c r="E81">
-        <v>779227.2188370905</v>
+        <v>779227.2188370909</v>
       </c>
     </row>
     <row r="82">
@@ -2191,10 +2191,10 @@
         </is>
       </c>
       <c r="D83">
-        <v>0.1495043919487083</v>
+        <v>0.1495043919487078</v>
       </c>
       <c r="E83">
-        <v>928356.8564953111</v>
+        <v>928356.8564953082</v>
       </c>
     </row>
     <row r="84">
@@ -2375,10 +2375,10 @@
         </is>
       </c>
       <c r="D91">
-        <v>0.1369334811613057</v>
+        <v>0.1369334811613063</v>
       </c>
       <c r="E91">
-        <v>850297.001063908</v>
+        <v>850297.0010639112</v>
       </c>
     </row>
     <row r="92">
@@ -2424,7 +2424,7 @@
         <v>0.15</v>
       </c>
       <c r="E93">
-        <v>931434.3656343658</v>
+        <v>931434.3656343656</v>
       </c>
     </row>
     <row r="94">
@@ -2467,10 +2467,10 @@
         </is>
       </c>
       <c r="D95">
-        <v>0.1130665188386942</v>
+        <v>0.1130665188386939</v>
       </c>
       <c r="E95">
-        <v>702093.6083267014</v>
+        <v>702093.6083266995</v>
       </c>
     </row>
     <row r="96">
@@ -2559,10 +2559,10 @@
         </is>
       </c>
       <c r="D99">
-        <v>0.0979014944789439</v>
+        <v>0.09790149447894382</v>
       </c>
       <c r="E99">
-        <v>607925.4426976766</v>
+        <v>607925.442697676</v>
       </c>
     </row>
     <row r="100">
@@ -2654,7 +2654,7 @@
         <v>0.1069382666493139</v>
       </c>
       <c r="E103">
-        <v>664039.8437236159</v>
+        <v>664039.8437236155</v>
       </c>
     </row>
     <row r="104">
@@ -2700,7 +2700,7 @@
         <v>0.15</v>
       </c>
       <c r="E105">
-        <v>931434.3656343656</v>
+        <v>931434.3656343658</v>
       </c>
     </row>
     <row r="106">
@@ -2789,10 +2789,10 @@
         </is>
       </c>
       <c r="D109">
-        <v>0.04516023887174229</v>
+        <v>0.04516023887174237</v>
       </c>
       <c r="E109">
-        <v>280425.322969318</v>
+        <v>280425.3229693185</v>
       </c>
     </row>
     <row r="110">
@@ -2812,10 +2812,10 @@
         </is>
       </c>
       <c r="D110">
-        <v>0.1397794007025374</v>
+        <v>0.1397794007025375</v>
       </c>
       <c r="E110">
-        <v>867968.9161474651</v>
+        <v>867968.9161474658</v>
       </c>
     </row>
     <row r="111">
@@ -2858,10 +2858,10 @@
         </is>
       </c>
       <c r="D112">
-        <v>0.04384650130868698</v>
+        <v>0.04384650130868686</v>
       </c>
       <c r="E112">
-        <v>272267.587544955</v>
+        <v>272267.5875449542</v>
       </c>
     </row>
     <row r="113">
@@ -3019,10 +3019,10 @@
         </is>
       </c>
       <c r="D119">
-        <v>0.07725182281606743</v>
+        <v>0.0772518228160676</v>
       </c>
       <c r="E119">
-        <v>479700.0171918813</v>
+        <v>479700.0171918824</v>
       </c>
     </row>
     <row r="120">
@@ -3367,7 +3367,7 @@
         <v>0.15</v>
       </c>
       <c r="E134">
-        <v>984549.0241900955</v>
+        <v>984549.0241900954</v>
       </c>
     </row>
     <row r="135">
@@ -3390,7 +3390,7 @@
         <v>0.15</v>
       </c>
       <c r="E135">
-        <v>984549.0241900954</v>
+        <v>984549.0241900955</v>
       </c>
     </row>
     <row r="136">
@@ -3410,10 +3410,10 @@
         </is>
       </c>
       <c r="D136">
-        <v>0.0400285575576973</v>
+        <v>0.04002855755769659</v>
       </c>
       <c r="E136">
-        <v>262733.848554453</v>
+        <v>262733.8485544483</v>
       </c>
     </row>
     <row r="137">
@@ -3456,10 +3456,10 @@
         </is>
       </c>
       <c r="D138">
-        <v>0.09884884927990978</v>
+        <v>0.09884884927991082</v>
       </c>
       <c r="E138">
-        <v>648810.2540056601</v>
+        <v>648810.2540056668</v>
       </c>
     </row>
     <row r="139">
@@ -3479,10 +3479,10 @@
         </is>
       </c>
       <c r="D139">
-        <v>0.1378497550084148</v>
+        <v>0.1378497550084149</v>
       </c>
       <c r="E139">
-        <v>904798.94518919</v>
+        <v>904798.9451891907</v>
       </c>
     </row>
     <row r="140">
@@ -3525,10 +3525,10 @@
         </is>
       </c>
       <c r="D141">
-        <v>0.1329556081264811</v>
+        <v>0.1329556081264807</v>
       </c>
       <c r="E141">
-        <v>872675.4282768511</v>
+        <v>872675.4282768487</v>
       </c>
     </row>
     <row r="142">
@@ -3571,10 +3571,10 @@
         </is>
       </c>
       <c r="D143">
-        <v>0.1403172300274972</v>
+        <v>0.1403172300274971</v>
       </c>
       <c r="E143">
-        <v>920994.6126708634</v>
+        <v>920994.6126708632</v>
       </c>
     </row>
     <row r="144">
@@ -3755,10 +3755,10 @@
         </is>
       </c>
       <c r="D151">
-        <v>0.1422973941192904</v>
+        <v>0.1422973941192908</v>
       </c>
       <c r="E151">
-        <v>933991.7368329387</v>
+        <v>933991.7368329415</v>
       </c>
     </row>
     <row r="152">
@@ -3847,10 +3847,10 @@
         </is>
       </c>
       <c r="D155">
-        <v>0.1077026058807096</v>
+        <v>0.1077026058807092</v>
       </c>
       <c r="E155">
-        <v>706923.303483887</v>
+        <v>706923.3034838844</v>
       </c>
     </row>
     <row r="156">
@@ -3939,10 +3939,10 @@
         </is>
       </c>
       <c r="D159">
-        <v>0.0979014944789439</v>
+        <v>0.09790149447894382</v>
       </c>
       <c r="E159">
-        <v>642592.139039975</v>
+        <v>642592.1390399744</v>
       </c>
     </row>
     <row r="160">
@@ -4034,7 +4034,7 @@
         <v>0.1069382666493139</v>
       </c>
       <c r="E163">
-        <v>701906.4405210818</v>
+        <v>701906.4405210814</v>
       </c>
     </row>
     <row r="164">
@@ -4080,7 +4080,7 @@
         <v>0.15</v>
       </c>
       <c r="E165">
-        <v>984549.0241900954</v>
+        <v>984549.0241900955</v>
       </c>
     </row>
     <row r="166">
@@ -4169,10 +4169,10 @@
         </is>
       </c>
       <c r="D169">
-        <v>0.04516023887174229</v>
+        <v>0.04516023887174237</v>
       </c>
       <c r="E169">
-        <v>296416.46075577</v>
+        <v>296416.4607557705</v>
       </c>
     </row>
     <row r="170">
@@ -4195,7 +4195,7 @@
         <v>0.1340148799990832</v>
       </c>
       <c r="E170">
-        <v>879628.1288670009</v>
+        <v>879628.1288670005</v>
       </c>
     </row>
     <row r="171">
@@ -4238,10 +4238,10 @@
         </is>
       </c>
       <c r="D172">
-        <v>0.04389186522681274</v>
+        <v>0.04389186522681283</v>
       </c>
       <c r="E172">
-        <v>288091.2871929444</v>
+        <v>288091.2871929451</v>
       </c>
     </row>
     <row r="173">
@@ -4307,10 +4307,10 @@
         </is>
       </c>
       <c r="D175">
-        <v>0.1432583966321582</v>
+        <v>0.1432583966321581</v>
       </c>
       <c r="E175">
-        <v>940299.4307415267</v>
+        <v>940299.430741526</v>
       </c>
     </row>
     <row r="176">
@@ -4356,7 +4356,7 @@
         <v>0.15</v>
       </c>
       <c r="E177">
-        <v>984549.0241900954</v>
+        <v>984549.0241900955</v>
       </c>
     </row>
     <row r="178">
@@ -4376,10 +4376,10 @@
         </is>
       </c>
       <c r="D178">
-        <v>0.004961888410446565</v>
+        <v>0.004961888410446552</v>
       </c>
       <c r="E178">
-        <v>32568.14928430207</v>
+        <v>32568.14928430198</v>
       </c>
     </row>
     <row r="179">
@@ -4399,10 +4399,10 @@
         </is>
       </c>
       <c r="D179">
-        <v>0.07387296973149943</v>
+        <v>0.07387296973149954</v>
       </c>
       <c r="E179">
-        <v>484877.0684211482</v>
+        <v>484877.0684211489</v>
       </c>
     </row>
     <row r="180">
@@ -4664,16 +4664,16 @@
         <v>0.1190553560393118</v>
       </c>
       <c r="G4">
-        <v>0.1446243886444422</v>
+        <v>0.1446243886444421</v>
       </c>
       <c r="H4">
-        <v>0.1446243886444422</v>
+        <v>0.1446243886444421</v>
       </c>
       <c r="I4">
-        <v>0.141684172237517</v>
+        <v>0.1416841722375169</v>
       </c>
       <c r="J4">
-        <v>0.05334769690189983</v>
+        <v>0.05334769690189982</v>
       </c>
       <c r="K4">
         <v>0.05368795891467298</v>
@@ -4684,7 +4684,7 @@
         </is>
       </c>
       <c r="M4">
-        <v>1</v>
+        <v>0.9999999999999999</v>
       </c>
     </row>
     <row r="5">
@@ -4722,7 +4722,7 @@
         <v>0.1246034918107483</v>
       </c>
       <c r="J5">
-        <v>0.04937366583187003</v>
+        <v>0.04937366583187001</v>
       </c>
       <c r="K5">
         <v>0.05008440219153319</v>
@@ -4823,7 +4823,7 @@
         <v>0.05332870461221242</v>
       </c>
       <c r="K7">
-        <v>0.05334121007677503</v>
+        <v>0.05334121007677502</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
@@ -4857,22 +4857,22 @@
         </is>
       </c>
       <c r="F8">
-        <v>0.1204819431658787</v>
+        <v>0.1204819431658786</v>
       </c>
       <c r="G8">
-        <v>0.1498265105424777</v>
+        <v>0.1498265105424776</v>
       </c>
       <c r="H8">
-        <v>0.1498265105424777</v>
+        <v>0.1498265105424776</v>
       </c>
       <c r="I8">
         <v>0.1497469326531883</v>
       </c>
       <c r="J8">
-        <v>0.0533287177921823</v>
+        <v>0.05332871779218228</v>
       </c>
       <c r="K8">
-        <v>0.05333829296211987</v>
+        <v>0.05333829296211985</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
@@ -4880,7 +4880,7 @@
         </is>
       </c>
       <c r="M8">
-        <v>0.9999999999999999</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -4906,7 +4906,7 @@
         </is>
       </c>
       <c r="F9">
-        <v>0.1190601279604179</v>
+        <v>0.119060127960418</v>
       </c>
       <c r="G9">
         <v>0.1446382300670524</v>
@@ -4929,7 +4929,7 @@
         </is>
       </c>
       <c r="M9">
-        <v>0.9999999999999999</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -5068,7 +5068,7 @@
         <v>0.05582678455974359</v>
       </c>
       <c r="K12">
-        <v>0.05584075692748226</v>
+        <v>0.05584075692748225</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
@@ -5117,7 +5117,7 @@
         <v>0.05583059394045162</v>
       </c>
       <c r="K13">
-        <v>0.05589744623857982</v>
+        <v>0.05589744623857983</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
@@ -5160,10 +5160,10 @@
         <v>0.1444114755701646</v>
       </c>
       <c r="I14">
-        <v>0.1413450253027814</v>
+        <v>0.1413450253027813</v>
       </c>
       <c r="J14">
-        <v>0.05571906749289481</v>
+        <v>0.05571906749289482</v>
       </c>
       <c r="K14">
         <v>0.05611230323574795</v>
@@ -5212,10 +5212,10 @@
         <v>0.1246034918107483</v>
       </c>
       <c r="J15">
-        <v>0.05162906558905112</v>
+        <v>0.05162906558905111</v>
       </c>
       <c r="K15">
-        <v>0.05241816121956138</v>
+        <v>0.05241816121956137</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
@@ -5261,10 +5261,10 @@
         <v>0.1394544991231728</v>
       </c>
       <c r="J16">
-        <v>0.04645652414139102</v>
+        <v>0.04645652414139103</v>
       </c>
       <c r="K16">
-        <v>0.04721328186405994</v>
+        <v>0.04721328186405996</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Publish committee memo and final submission files
</commit_message>
<xml_diff>
--- a/portfolio_construction/Portfolio Final/Results.xlsx
+++ b/portfolio_construction/Portfolio Final/Results.xlsx
@@ -995,10 +995,10 @@
         </is>
       </c>
       <c r="D31">
-        <v>0.1372476690650976</v>
+        <v>0.1372476690650974</v>
       </c>
       <c r="E31">
-        <v>854949.5969144441</v>
+        <v>854949.5969144428</v>
       </c>
     </row>
     <row r="32">
@@ -1087,10 +1087,10 @@
         </is>
       </c>
       <c r="D35">
-        <v>0.1127523309349023</v>
+        <v>0.1127523309349027</v>
       </c>
       <c r="E35">
-        <v>702362.0913972433</v>
+        <v>702362.091397246</v>
       </c>
     </row>
     <row r="36">
@@ -1179,10 +1179,10 @@
         </is>
       </c>
       <c r="D39">
-        <v>0.09790149447894382</v>
+        <v>0.0979014944789439</v>
       </c>
       <c r="E39">
-        <v>609852.5666209657</v>
+        <v>609852.5666209663</v>
       </c>
     </row>
     <row r="40">
@@ -1274,7 +1274,7 @@
         <v>0.1069382666493139</v>
       </c>
       <c r="E43">
-        <v>666144.850323074</v>
+        <v>666144.8503230744</v>
       </c>
     </row>
     <row r="44">
@@ -1320,7 +1320,7 @@
         <v>0.15</v>
       </c>
       <c r="E45">
-        <v>934387.012987013</v>
+        <v>934387.0129870129</v>
       </c>
     </row>
     <row r="46">
@@ -1409,10 +1409,10 @@
         </is>
       </c>
       <c r="D49">
-        <v>0.04516023887174237</v>
+        <v>0.04516023887174229</v>
       </c>
       <c r="E49">
-        <v>281314.271367649</v>
+        <v>281314.2713676485</v>
       </c>
     </row>
     <row r="50">
@@ -1478,10 +1478,10 @@
         </is>
       </c>
       <c r="D52">
-        <v>0.04391359239887393</v>
+        <v>0.04391359239887407</v>
       </c>
       <c r="E52">
-        <v>273548.6028740867</v>
+        <v>273548.6028740876</v>
       </c>
     </row>
     <row r="53">
@@ -1550,7 +1550,7 @@
         <v>0.1393715969982425</v>
       </c>
       <c r="E55">
-        <v>868180.0680961172</v>
+        <v>868180.0680961171</v>
       </c>
     </row>
     <row r="56">
@@ -1616,10 +1616,10 @@
         </is>
       </c>
       <c r="D58">
-        <v>0.0001758333460199342</v>
+        <v>0.0001758333460199443</v>
       </c>
       <c r="E58">
-        <v>1095.309299807188</v>
+        <v>1095.309299807251</v>
       </c>
     </row>
     <row r="59">
@@ -1639,10 +1639,10 @@
         </is>
       </c>
       <c r="D59">
-        <v>0.07708630041242333</v>
+        <v>0.07708630041242337</v>
       </c>
       <c r="E59">
-        <v>480189.5865638919</v>
+        <v>480189.5865638921</v>
       </c>
     </row>
     <row r="60">
@@ -2007,10 +2007,10 @@
         </is>
       </c>
       <c r="D75">
-        <v>0.1499999999999999</v>
+        <v>0.15</v>
       </c>
       <c r="E75">
-        <v>931434.3656343655</v>
+        <v>931434.3656343658</v>
       </c>
     </row>
     <row r="76">
@@ -2030,10 +2030,10 @@
         </is>
       </c>
       <c r="D76">
-        <v>0.04257117849736258</v>
+        <v>0.04257117849736252</v>
       </c>
       <c r="E76">
-        <v>264348.3909199885</v>
+        <v>264348.3909199881</v>
       </c>
     </row>
     <row r="77">
@@ -2076,10 +2076,10 @@
         </is>
       </c>
       <c r="D78">
-        <v>0.09048938186563847</v>
+        <v>0.09048938186563894</v>
       </c>
       <c r="E78">
-        <v>561899.4666311124</v>
+        <v>561899.4666311153</v>
       </c>
     </row>
     <row r="79">
@@ -2099,10 +2099,10 @@
         </is>
       </c>
       <c r="D79">
-        <v>0.1419467823439498</v>
+        <v>0.1419467823439489</v>
       </c>
       <c r="E79">
-        <v>881427.4077758415</v>
+        <v>881427.4077758364</v>
       </c>
     </row>
     <row r="80">
@@ -2148,7 +2148,7 @@
         <v>0.1254882653443414</v>
       </c>
       <c r="E81">
-        <v>779227.2188370909</v>
+        <v>779227.2188370905</v>
       </c>
     </row>
     <row r="82">
@@ -2191,10 +2191,10 @@
         </is>
       </c>
       <c r="D83">
-        <v>0.1495043919487078</v>
+        <v>0.1495043919487083</v>
       </c>
       <c r="E83">
-        <v>928356.8564953082</v>
+        <v>928356.8564953111</v>
       </c>
     </row>
     <row r="84">
@@ -2375,10 +2375,10 @@
         </is>
       </c>
       <c r="D91">
-        <v>0.1369334811613063</v>
+        <v>0.1369334811613057</v>
       </c>
       <c r="E91">
-        <v>850297.0010639112</v>
+        <v>850297.001063908</v>
       </c>
     </row>
     <row r="92">
@@ -2424,7 +2424,7 @@
         <v>0.15</v>
       </c>
       <c r="E93">
-        <v>931434.3656343656</v>
+        <v>931434.3656343658</v>
       </c>
     </row>
     <row r="94">
@@ -2467,10 +2467,10 @@
         </is>
       </c>
       <c r="D95">
-        <v>0.1130665188386939</v>
+        <v>0.1130665188386942</v>
       </c>
       <c r="E95">
-        <v>702093.6083266995</v>
+        <v>702093.6083267014</v>
       </c>
     </row>
     <row r="96">
@@ -2559,10 +2559,10 @@
         </is>
       </c>
       <c r="D99">
-        <v>0.09790149447894382</v>
+        <v>0.0979014944789439</v>
       </c>
       <c r="E99">
-        <v>607925.442697676</v>
+        <v>607925.4426976766</v>
       </c>
     </row>
     <row r="100">
@@ -2654,7 +2654,7 @@
         <v>0.1069382666493139</v>
       </c>
       <c r="E103">
-        <v>664039.8437236155</v>
+        <v>664039.8437236159</v>
       </c>
     </row>
     <row r="104">
@@ -2700,7 +2700,7 @@
         <v>0.15</v>
       </c>
       <c r="E105">
-        <v>931434.3656343658</v>
+        <v>931434.3656343656</v>
       </c>
     </row>
     <row r="106">
@@ -2789,10 +2789,10 @@
         </is>
       </c>
       <c r="D109">
-        <v>0.04516023887174237</v>
+        <v>0.04516023887174229</v>
       </c>
       <c r="E109">
-        <v>280425.3229693185</v>
+        <v>280425.322969318</v>
       </c>
     </row>
     <row r="110">
@@ -2812,10 +2812,10 @@
         </is>
       </c>
       <c r="D110">
-        <v>0.1397794007025375</v>
+        <v>0.1397794007025374</v>
       </c>
       <c r="E110">
-        <v>867968.9161474658</v>
+        <v>867968.9161474651</v>
       </c>
     </row>
     <row r="111">
@@ -2858,10 +2858,10 @@
         </is>
       </c>
       <c r="D112">
-        <v>0.04384650130868686</v>
+        <v>0.04384650130868698</v>
       </c>
       <c r="E112">
-        <v>272267.5875449542</v>
+        <v>272267.587544955</v>
       </c>
     </row>
     <row r="113">
@@ -3019,10 +3019,10 @@
         </is>
       </c>
       <c r="D119">
-        <v>0.0772518228160676</v>
+        <v>0.07725182281606743</v>
       </c>
       <c r="E119">
-        <v>479700.0171918824</v>
+        <v>479700.0171918813</v>
       </c>
     </row>
     <row r="120">
@@ -3367,7 +3367,7 @@
         <v>0.15</v>
       </c>
       <c r="E134">
-        <v>984549.0241900954</v>
+        <v>984549.0241900955</v>
       </c>
     </row>
     <row r="135">
@@ -3390,7 +3390,7 @@
         <v>0.15</v>
       </c>
       <c r="E135">
-        <v>984549.0241900955</v>
+        <v>984549.0241900954</v>
       </c>
     </row>
     <row r="136">
@@ -3410,10 +3410,10 @@
         </is>
       </c>
       <c r="D136">
-        <v>0.04002855755769659</v>
+        <v>0.0400285575576973</v>
       </c>
       <c r="E136">
-        <v>262733.8485544483</v>
+        <v>262733.848554453</v>
       </c>
     </row>
     <row r="137">
@@ -3456,10 +3456,10 @@
         </is>
       </c>
       <c r="D138">
-        <v>0.09884884927991082</v>
+        <v>0.09884884927990978</v>
       </c>
       <c r="E138">
-        <v>648810.2540056668</v>
+        <v>648810.2540056601</v>
       </c>
     </row>
     <row r="139">
@@ -3479,10 +3479,10 @@
         </is>
       </c>
       <c r="D139">
-        <v>0.1378497550084149</v>
+        <v>0.1378497550084148</v>
       </c>
       <c r="E139">
-        <v>904798.9451891907</v>
+        <v>904798.94518919</v>
       </c>
     </row>
     <row r="140">
@@ -3525,10 +3525,10 @@
         </is>
       </c>
       <c r="D141">
-        <v>0.1329556081264807</v>
+        <v>0.1329556081264811</v>
       </c>
       <c r="E141">
-        <v>872675.4282768487</v>
+        <v>872675.4282768511</v>
       </c>
     </row>
     <row r="142">
@@ -3571,10 +3571,10 @@
         </is>
       </c>
       <c r="D143">
-        <v>0.1403172300274971</v>
+        <v>0.1403172300274972</v>
       </c>
       <c r="E143">
-        <v>920994.6126708632</v>
+        <v>920994.6126708634</v>
       </c>
     </row>
     <row r="144">
@@ -3755,10 +3755,10 @@
         </is>
       </c>
       <c r="D151">
-        <v>0.1422973941192908</v>
+        <v>0.1422973941192904</v>
       </c>
       <c r="E151">
-        <v>933991.7368329415</v>
+        <v>933991.7368329387</v>
       </c>
     </row>
     <row r="152">
@@ -3847,10 +3847,10 @@
         </is>
       </c>
       <c r="D155">
-        <v>0.1077026058807092</v>
+        <v>0.1077026058807096</v>
       </c>
       <c r="E155">
-        <v>706923.3034838844</v>
+        <v>706923.303483887</v>
       </c>
     </row>
     <row r="156">
@@ -3939,10 +3939,10 @@
         </is>
       </c>
       <c r="D159">
-        <v>0.09790149447894382</v>
+        <v>0.0979014944789439</v>
       </c>
       <c r="E159">
-        <v>642592.1390399744</v>
+        <v>642592.139039975</v>
       </c>
     </row>
     <row r="160">
@@ -4034,7 +4034,7 @@
         <v>0.1069382666493139</v>
       </c>
       <c r="E163">
-        <v>701906.4405210814</v>
+        <v>701906.4405210818</v>
       </c>
     </row>
     <row r="164">
@@ -4080,7 +4080,7 @@
         <v>0.15</v>
       </c>
       <c r="E165">
-        <v>984549.0241900955</v>
+        <v>984549.0241900954</v>
       </c>
     </row>
     <row r="166">
@@ -4169,10 +4169,10 @@
         </is>
       </c>
       <c r="D169">
-        <v>0.04516023887174237</v>
+        <v>0.04516023887174229</v>
       </c>
       <c r="E169">
-        <v>296416.4607557705</v>
+        <v>296416.46075577</v>
       </c>
     </row>
     <row r="170">
@@ -4195,7 +4195,7 @@
         <v>0.1340148799990832</v>
       </c>
       <c r="E170">
-        <v>879628.1288670005</v>
+        <v>879628.1288670009</v>
       </c>
     </row>
     <row r="171">
@@ -4238,10 +4238,10 @@
         </is>
       </c>
       <c r="D172">
-        <v>0.04389186522681283</v>
+        <v>0.04389186522681274</v>
       </c>
       <c r="E172">
-        <v>288091.2871929451</v>
+        <v>288091.2871929444</v>
       </c>
     </row>
     <row r="173">
@@ -4307,10 +4307,10 @@
         </is>
       </c>
       <c r="D175">
-        <v>0.1432583966321581</v>
+        <v>0.1432583966321582</v>
       </c>
       <c r="E175">
-        <v>940299.430741526</v>
+        <v>940299.4307415267</v>
       </c>
     </row>
     <row r="176">
@@ -4356,7 +4356,7 @@
         <v>0.15</v>
       </c>
       <c r="E177">
-        <v>984549.0241900955</v>
+        <v>984549.0241900954</v>
       </c>
     </row>
     <row r="178">
@@ -4376,10 +4376,10 @@
         </is>
       </c>
       <c r="D178">
-        <v>0.004961888410446552</v>
+        <v>0.004961888410446565</v>
       </c>
       <c r="E178">
-        <v>32568.14928430198</v>
+        <v>32568.14928430207</v>
       </c>
     </row>
     <row r="179">
@@ -4399,10 +4399,10 @@
         </is>
       </c>
       <c r="D179">
-        <v>0.07387296973149954</v>
+        <v>0.07387296973149943</v>
       </c>
       <c r="E179">
-        <v>484877.0684211489</v>
+        <v>484877.0684211482</v>
       </c>
     </row>
     <row r="180">
@@ -4664,16 +4664,16 @@
         <v>0.1190553560393118</v>
       </c>
       <c r="G4">
-        <v>0.1446243886444421</v>
+        <v>0.1446243886444422</v>
       </c>
       <c r="H4">
-        <v>0.1446243886444421</v>
+        <v>0.1446243886444422</v>
       </c>
       <c r="I4">
-        <v>0.1416841722375169</v>
+        <v>0.141684172237517</v>
       </c>
       <c r="J4">
-        <v>0.05334769690189982</v>
+        <v>0.05334769690189983</v>
       </c>
       <c r="K4">
         <v>0.05368795891467298</v>
@@ -4684,7 +4684,7 @@
         </is>
       </c>
       <c r="M4">
-        <v>0.9999999999999999</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -4722,7 +4722,7 @@
         <v>0.1246034918107483</v>
       </c>
       <c r="J5">
-        <v>0.04937366583187001</v>
+        <v>0.04937366583187003</v>
       </c>
       <c r="K5">
         <v>0.05008440219153319</v>
@@ -4823,7 +4823,7 @@
         <v>0.05332870461221242</v>
       </c>
       <c r="K7">
-        <v>0.05334121007677502</v>
+        <v>0.05334121007677503</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
@@ -4857,22 +4857,22 @@
         </is>
       </c>
       <c r="F8">
-        <v>0.1204819431658786</v>
+        <v>0.1204819431658787</v>
       </c>
       <c r="G8">
-        <v>0.1498265105424776</v>
+        <v>0.1498265105424777</v>
       </c>
       <c r="H8">
-        <v>0.1498265105424776</v>
+        <v>0.1498265105424777</v>
       </c>
       <c r="I8">
         <v>0.1497469326531883</v>
       </c>
       <c r="J8">
-        <v>0.05332871779218228</v>
+        <v>0.0533287177921823</v>
       </c>
       <c r="K8">
-        <v>0.05333829296211985</v>
+        <v>0.05333829296211987</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
@@ -4880,7 +4880,7 @@
         </is>
       </c>
       <c r="M8">
-        <v>1</v>
+        <v>0.9999999999999999</v>
       </c>
     </row>
     <row r="9">
@@ -4906,7 +4906,7 @@
         </is>
       </c>
       <c r="F9">
-        <v>0.119060127960418</v>
+        <v>0.1190601279604179</v>
       </c>
       <c r="G9">
         <v>0.1446382300670524</v>
@@ -4929,7 +4929,7 @@
         </is>
       </c>
       <c r="M9">
-        <v>1</v>
+        <v>0.9999999999999999</v>
       </c>
     </row>
     <row r="10">
@@ -5068,7 +5068,7 @@
         <v>0.05582678455974359</v>
       </c>
       <c r="K12">
-        <v>0.05584075692748225</v>
+        <v>0.05584075692748226</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
@@ -5117,7 +5117,7 @@
         <v>0.05583059394045162</v>
       </c>
       <c r="K13">
-        <v>0.05589744623857983</v>
+        <v>0.05589744623857982</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
@@ -5160,10 +5160,10 @@
         <v>0.1444114755701646</v>
       </c>
       <c r="I14">
-        <v>0.1413450253027813</v>
+        <v>0.1413450253027814</v>
       </c>
       <c r="J14">
-        <v>0.05571906749289482</v>
+        <v>0.05571906749289481</v>
       </c>
       <c r="K14">
         <v>0.05611230323574795</v>
@@ -5212,10 +5212,10 @@
         <v>0.1246034918107483</v>
       </c>
       <c r="J15">
-        <v>0.05162906558905111</v>
+        <v>0.05162906558905112</v>
       </c>
       <c r="K15">
-        <v>0.05241816121956137</v>
+        <v>0.05241816121956138</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
@@ -5261,10 +5261,10 @@
         <v>0.1394544991231728</v>
       </c>
       <c r="J16">
-        <v>0.04645652414139103</v>
+        <v>0.04645652414139102</v>
       </c>
       <c r="K16">
-        <v>0.04721328186405996</v>
+        <v>0.04721328186405994</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>

</xml_diff>